<commit_message>
Switch to priced per-item product photos
Gavin supplied 4 photos per product type ranked cheapest (1) to most
expensive (4). Each catalog item now shows its own photo matched by
actual price rank within its product type (verified programmatically,
since row order didn't always match price order), instead of one
photo shared across all variants of a product type.

Also resolves a missing/duplicate tier-number conflict for Butter,
Canned Tuna, and Cheddar Cheese (confirmed with Gavin), and drops
Yogurt's two "vanilla" variants so it matches the standard 4-variant
pattern every other product type follows (Gavin's call, since there
were only 4 numbered yogurt photos for 6 catalog variants).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog-design.xlsx
+++ b/catalog-design.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalog'!$A$1:$K$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalog'!$A$1:$K$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2472,7 +2472,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>yogurt-sb-vanilla</t>
+          <t>yogurt-sb-organic-plain</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Vanilla Yogurt (32 oz)</t>
+          <t>EveryDay Basics Organic Plain Yogurt (32 oz)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Conventional Dairy</t>
+          <t>Pasture-Raised</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2515,19 +2515,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J36" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K36" s="5" t="n">
-        <v>3.79</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>yogurt-brand-vanilla</t>
+          <t>yogurt-brand-organic-plain</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Green Pasture Co. Vanilla Yogurt (32 oz)</t>
+          <t>Green Pasture Co. Organic Plain Yogurt (32 oz)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2557,12 +2557,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Conventional Dairy</t>
+          <t>Pasture-Raised</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2570,19 +2570,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="J37" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K37" s="5" t="n">
-        <v>5.29</v>
+        <v>6.99</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>yogurt-sb-organic-plain</t>
+          <t>butter-sb-conv</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
@@ -2592,12 +2592,12 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Yogurt</t>
+          <t>Butter</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Organic Plain Yogurt (32 oz)</t>
+          <t>EveryDay Basics Butter (1 lb)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -2612,32 +2612,32 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Pasture-Raised</t>
+          <t>Conventional Dairy</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J38" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+          <t>USA (Wisconsin)</t>
+        </is>
+      </c>
+      <c r="J38" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K38" s="5" t="n">
-        <v>5.49</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>yogurt-brand-organic-plain</t>
+          <t>butter-brand-conv</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
@@ -2647,12 +2647,12 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Yogurt</t>
+          <t>Butter</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Green Pasture Co. Organic Plain Yogurt (32 oz)</t>
+          <t>Green Pasture Co. Butter (1 lb)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2667,32 +2667,32 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Pasture-Raised</t>
+          <t>Conventional Dairy</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+          <t>USA (Wisconsin)</t>
+        </is>
+      </c>
+      <c r="J39" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K39" s="5" t="n">
-        <v>6.99</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>butter-sb-conv</t>
+          <t>butter-sb-organic</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Butter (1 lb)</t>
+          <t>EveryDay Basics Organic Butter (1 lb)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2722,17 +2722,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Conventional Dairy</t>
+          <t>Pasture-Raised</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>USA (Wisconsin)</t>
+          <t>USA (Vermont)</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr">
@@ -2741,13 +2741,13 @@
         </is>
       </c>
       <c r="K40" s="5" t="n">
-        <v>3.99</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>butter-brand-conv</t>
+          <t>butter-brand-organic</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Green Pasture Co. Butter (1 lb)</t>
+          <t>Green Pasture Co. Organic Grass-Fed Butter (1 lb)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -2777,17 +2777,17 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Conventional Dairy</t>
+          <t>Pasture-Raised/Grass-Fed</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>USA (Wisconsin)</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="J41" s="9" t="inlineStr">
@@ -2796,28 +2796,28 @@
         </is>
       </c>
       <c r="K41" s="5" t="n">
-        <v>5.49</v>
+        <v>7.99</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>butter-sb-organic</t>
+          <t>chicken-sb-factory</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Dairy &amp; Eggs</t>
+          <t>Meat &amp; Seafood</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Chicken Breast</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Organic Butter (1 lb)</t>
+          <t>EveryDay Basics Chicken Breast (1 lb)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2832,52 +2832,52 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Pasture-Raised</t>
+          <t>Factory-Farmed</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>USA (Vermont)</t>
-        </is>
-      </c>
-      <c r="J42" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+          <t>USA (Arkansas)</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K42" s="5" t="n">
-        <v>6.49</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>butter-brand-organic</t>
+          <t>chicken-brand-factory</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Dairy &amp; Eggs</t>
+          <t>Meat &amp; Seafood</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Butter</t>
+          <t>Chicken Breast</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Green Pasture Co. Organic Grass-Fed Butter (1 lb)</t>
+          <t>Heritage Range Chicken Breast (1 lb)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Green Pasture Co.</t>
+          <t>Heritage Range</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -2887,32 +2887,32 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Pasture-Raised/Grass-Fed</t>
+          <t>Factory-Farmed</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-      <c r="J43" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+          <t>USA (Arkansas)</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K43" s="5" t="n">
-        <v>7.99</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>chicken-sb-factory</t>
+          <t>chicken-sb-freerange</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Chicken Breast (1 lb)</t>
+          <t>EveryDay Basics Free-Range Chicken Breast (1 lb)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2947,12 +2947,12 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Factory-Farmed</t>
+          <t>Free-Range</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>USA (Arkansas)</t>
+          <t>USA (Pennsylvania)</t>
         </is>
       </c>
       <c r="J44" s="4" t="inlineStr">
@@ -2961,13 +2961,13 @@
         </is>
       </c>
       <c r="K44" s="5" t="n">
-        <v>3.99</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>chicken-brand-factory</t>
+          <t>chicken-brand-freerange-org</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Chicken Breast (1 lb)</t>
+          <t>Heritage Range Organic Free-Range Chicken Breast (1 lb)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
@@ -2997,17 +2997,17 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Factory-Farmed</t>
+          <t>Free-Range</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>USA (Arkansas)</t>
+          <t>USA (Pennsylvania)</t>
         </is>
       </c>
       <c r="J45" s="4" t="inlineStr">
@@ -3016,13 +3016,13 @@
         </is>
       </c>
       <c r="K45" s="5" t="n">
-        <v>4.99</v>
+        <v>8.99</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>chicken-sb-freerange</t>
+          <t>beef-sb-factory</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3032,12 +3032,12 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Chicken Breast</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Free-Range Chicken Breast (1 lb)</t>
+          <t>EveryDay Basics Ground Beef 80/20 (1 lb)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -3057,27 +3057,27 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Free-Range</t>
+          <t>Factory-Farmed (Grain-Fed)</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>USA (Pennsylvania)</t>
-        </is>
-      </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>USA (Nebraska)</t>
+        </is>
+      </c>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K46" s="5" t="n">
-        <v>6.49</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>chicken-brand-freerange-org</t>
+          <t>beef-brand-factory</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -3087,12 +3087,12 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Chicken Breast</t>
+          <t>Ground Beef</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Organic Free-Range Chicken Breast (1 lb)</t>
+          <t>Heritage Range Ground Beef 80/20 (1 lb)</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -3107,32 +3107,32 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Free-Range</t>
+          <t>Factory-Farmed (Grain-Fed)</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>USA (Pennsylvania)</t>
-        </is>
-      </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>USA (Nebraska)</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K47" s="5" t="n">
-        <v>8.99</v>
+        <v>6.99</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>beef-sb-factory</t>
+          <t>beef-sb-grassfed</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Ground Beef 80/20 (1 lb)</t>
+          <t>EveryDay Basics Grass-Fed Ground Beef (1 lb)</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -3167,12 +3167,12 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Factory-Farmed (Grain-Fed)</t>
+          <t>Grass-Fed/Pasture-Raised</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>USA (Nebraska)</t>
+          <t>USA (Montana)</t>
         </is>
       </c>
       <c r="J48" s="7" t="inlineStr">
@@ -3181,13 +3181,13 @@
         </is>
       </c>
       <c r="K48" s="5" t="n">
-        <v>5.49</v>
+        <v>8.49</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>beef-brand-factory</t>
+          <t>beef-brand-grassfed-org</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -3202,7 +3202,7 @@
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Ground Beef 80/20 (1 lb)</t>
+          <t>Heritage Range Organic Grass-Fed Ground Beef (1 lb)</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
@@ -3217,17 +3217,17 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Factory-Farmed (Grain-Fed)</t>
+          <t>Grass-Fed/Pasture-Raised</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>USA (Nebraska)</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
@@ -3236,13 +3236,13 @@
         </is>
       </c>
       <c r="K49" s="5" t="n">
-        <v>6.99</v>
+        <v>10.99</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>beef-sb-grassfed</t>
+          <t>bacon-sb-factory</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -3252,12 +3252,12 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Bacon</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Grass-Fed Ground Beef (1 lb)</t>
+          <t>EveryDay Basics Bacon (12 oz)</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -3277,27 +3277,27 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Grass-Fed/Pasture-Raised</t>
+          <t>Factory-Farmed</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>USA (Montana)</t>
-        </is>
-      </c>
-      <c r="J50" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J50" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K50" s="5" t="n">
-        <v>8.49</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>beef-brand-grassfed-org</t>
+          <t>bacon-brand-factory</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -3307,12 +3307,12 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Ground Beef</t>
+          <t>Bacon</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Organic Grass-Fed Ground Beef (1 lb)</t>
+          <t>Heritage Range Bacon (12 oz)</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
@@ -3327,32 +3327,32 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>Grass-Fed/Pasture-Raised</t>
+          <t>Factory-Farmed</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-      <c r="J51" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J51" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K51" s="5" t="n">
-        <v>10.99</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>bacon-sb-factory</t>
+          <t>bacon-sb-freerange</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Bacon (12 oz)</t>
+          <t>EveryDay Basics Uncured Free-Range Bacon (12 oz)</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -3387,7 +3387,7 @@
       </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
-          <t>Factory-Farmed</t>
+          <t>Free-Range</t>
         </is>
       </c>
       <c r="I52" s="2" t="inlineStr">
@@ -3401,13 +3401,13 @@
         </is>
       </c>
       <c r="K52" s="5" t="n">
-        <v>4.99</v>
+        <v>7.99</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>bacon-brand-factory</t>
+          <t>bacon-brand-freerange-org</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -3422,7 +3422,7 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Bacon (12 oz)</t>
+          <t>Heritage Range Organic Free-Range Bacon (12 oz)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -3437,12 +3437,12 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>Factory-Farmed</t>
+          <t>Free-Range</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr">
@@ -3456,13 +3456,13 @@
         </is>
       </c>
       <c r="K53" s="5" t="n">
-        <v>6.49</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>bacon-sb-freerange</t>
+          <t>salmon-sb-farmed</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -3472,12 +3472,12 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Bacon</t>
+          <t>Salmon Fillet</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Uncured Free-Range Bacon (12 oz)</t>
+          <t>EveryDay Basics Salmon Fillet (1 lb)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -3497,17 +3497,17 @@
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>Free-Range</t>
+          <t>Farmed</t>
         </is>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>USA (Iowa)</t>
-        </is>
-      </c>
-      <c r="J54" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K54" s="5" t="n">
@@ -3517,7 +3517,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>bacon-brand-freerange-org</t>
+          <t>salmon-brand-farmed</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -3527,12 +3527,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Bacon</t>
+          <t>Salmon Fillet</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Organic Free-Range Bacon (12 oz)</t>
+          <t>Heritage Range Salmon Fillet (1 lb)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
@@ -3547,32 +3547,32 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>Free-Range</t>
+          <t>Farmed</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>USA (Iowa)</t>
-        </is>
-      </c>
-      <c r="J55" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K55" s="5" t="n">
-        <v>9.99</v>
+        <v>9.49</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>salmon-sb-farmed</t>
+          <t>salmon-sb-wild</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -3587,7 +3587,7 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Salmon Fillet (1 lb)</t>
+          <t>EveryDay Basics Wild-Caught Salmon Fillet (1 lb)</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -3607,12 +3607,12 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Farmed</t>
+          <t>Wild-Caught</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>USA (Alaska)</t>
         </is>
       </c>
       <c r="J56" s="4" t="inlineStr">
@@ -3621,13 +3621,13 @@
         </is>
       </c>
       <c r="K56" s="5" t="n">
-        <v>7.99</v>
+        <v>11.99</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>salmon-brand-farmed</t>
+          <t>salmon-brand-wild-msc</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -3642,7 +3642,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Salmon Fillet (1 lb)</t>
+          <t>Heritage Range Wild-Caught Salmon Fillet (1 lb)</t>
         </is>
       </c>
       <c r="E57" s="2" t="inlineStr">
@@ -3662,12 +3662,12 @@
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>Farmed</t>
+          <t>Wild-Caught, MSC Certified</t>
         </is>
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>USA (Alaska)</t>
         </is>
       </c>
       <c r="J57" s="4" t="inlineStr">
@@ -3676,13 +3676,13 @@
         </is>
       </c>
       <c r="K57" s="5" t="n">
-        <v>9.49</v>
+        <v>14.99</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>salmon-sb-wild</t>
+          <t>tuna-sb-std</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -3692,12 +3692,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Salmon Fillet</t>
+          <t>Canned Tuna</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Wild-Caught Salmon Fillet (1 lb)</t>
+          <t>EveryDay Basics Chunk Tuna in Water (5 oz)</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -3717,12 +3717,12 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Wild-Caught</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>USA (Alaska)</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="J58" s="4" t="inlineStr">
@@ -3731,13 +3731,13 @@
         </is>
       </c>
       <c r="K58" s="5" t="n">
-        <v>11.99</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>salmon-brand-wild-msc</t>
+          <t>tuna-brand-std</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -3747,17 +3747,17 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Salmon Fillet</t>
+          <t>Canned Tuna</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Heritage Range Wild-Caught Salmon Fillet (1 lb)</t>
+          <t>Pinnacle Foods Chunk Tuna in Water (5 oz)</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Heritage Range</t>
+          <t>Pinnacle Foods</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -3772,12 +3772,12 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>Wild-Caught, MSC Certified</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>USA (Alaska)</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="J59" s="4" t="inlineStr">
@@ -3786,13 +3786,13 @@
         </is>
       </c>
       <c r="K59" s="5" t="n">
-        <v>14.99</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>tuna-sb-std</t>
+          <t>tuna-sb-wild</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -3807,7 +3807,7 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Chunk Tuna in Water (5 oz)</t>
+          <t>EveryDay Basics Wild-Caught Tuna in Water (5 oz)</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -3827,12 +3827,12 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Wild-Caught, Dolphin-Safe</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="J60" s="4" t="inlineStr">
@@ -3841,13 +3841,13 @@
         </is>
       </c>
       <c r="K60" s="5" t="n">
-        <v>1.29</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>tuna-brand-std</t>
+          <t>tuna-brand-wild-oil</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3862,7 +3862,7 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Chunk Tuna in Water (5 oz)</t>
+          <t>Pinnacle Foods Wild-Caught Tuna in Olive Oil (5 oz)</t>
         </is>
       </c>
       <c r="E61" s="2" t="inlineStr">
@@ -3882,42 +3882,42 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Wild-Caught, Dolphin-Safe</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Thailand</t>
-        </is>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="J61" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K61" s="5" t="n">
-        <v>1.99</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>tuna-sb-wild</t>
+          <t>bread-sb-white</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Meat &amp; Seafood</t>
+          <t>Bakery &amp; Grains</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Canned Tuna</t>
+          <t>Bread</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Wild-Caught Tuna in Water (5 oz)</t>
+          <t>EveryDay Basics White Bread (24 oz loaf)</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -3937,7 +3937,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>Wild-Caught, Dolphin-Safe</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -3945,9 +3945,9 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J62" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K62" s="5" t="n">
@@ -3957,27 +3957,27 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>tuna-brand-wild-oil</t>
+          <t>bread-brand-white</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Meat &amp; Seafood</t>
+          <t>Bakery &amp; Grains</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Canned Tuna</t>
+          <t>Bread</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Wild-Caught Tuna in Olive Oil (5 oz)</t>
+          <t>Golden Harvest White Bread (24 oz loaf)</t>
         </is>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Pinnacle Foods</t>
+          <t>Golden Harvest</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -3992,17 +3992,17 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>Wild-Caught, Dolphin-Safe</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="J63" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K63" s="5" t="n">
@@ -4012,7 +4012,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>bread-sb-white</t>
+          <t>bread-sb-wheat</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics White Bread (24 oz loaf)</t>
+          <t>EveryDay Basics Whole Wheat Bread (24 oz loaf)</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -4055,19 +4055,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J64" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K64" s="5" t="n">
-        <v>2.49</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>bread-brand-white</t>
+          <t>bread-brand-wheat-org</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest White Bread (24 oz loaf)</t>
+          <t>Golden Harvest Organic Whole Wheat Bread (24 oz loaf)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -4110,19 +4110,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J65" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K65" s="5" t="n">
-        <v>3.49</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>bread-sb-wheat</t>
+          <t>pasta-sb-reg</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4132,12 +4132,12 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Bread</t>
+          <t>Pasta</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Whole Wheat Bread (24 oz loaf)</t>
+          <t>EveryDay Basics Spaghetti (1 lb box)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -4162,22 +4162,22 @@
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J66" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="J66" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K66" s="5" t="n">
-        <v>2.99</v>
+        <v>1.29</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>bread-brand-wheat-org</t>
+          <t>pasta-brand-reg</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -4187,12 +4187,12 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Bread</t>
+          <t>Pasta</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Organic Whole Wheat Bread (24 oz loaf)</t>
+          <t>Golden Harvest Spaghetti (1 lb box)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
@@ -4207,7 +4207,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -4217,22 +4217,22 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J67" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="J67" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K67" s="5" t="n">
-        <v>4.99</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>pasta-sb-reg</t>
+          <t>pasta-sb-wheat</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -4247,7 +4247,7 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Spaghetti (1 lb box)</t>
+          <t>EveryDay Basics Whole Wheat Spaghetti (1 lb box)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -4275,19 +4275,19 @@
           <t>Italy</t>
         </is>
       </c>
-      <c r="J68" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K68" s="5" t="n">
-        <v>1.29</v>
+        <v>1.79</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>pasta-brand-reg</t>
+          <t>pasta-brand-wheat-org</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Spaghetti (1 lb box)</t>
+          <t>Golden Harvest Organic Whole Wheat Spaghetti (1 lb box)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -4330,19 +4330,19 @@
           <t>Italy</t>
         </is>
       </c>
-      <c r="J69" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K69" s="5" t="n">
-        <v>1.99</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>pasta-sb-wheat</t>
+          <t>rice-sb-white</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -4352,12 +4352,12 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Pasta</t>
+          <t>Rice</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Whole Wheat Spaghetti (1 lb box)</t>
+          <t>EveryDay Basics White Rice (2 lb bag)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -4382,22 +4382,22 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="J70" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K70" s="5" t="n">
-        <v>1.79</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>pasta-brand-wheat-org</t>
+          <t>rice-brand-white</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -4407,12 +4407,12 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Pasta</t>
+          <t>Rice</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Organic Whole Wheat Spaghetti (1 lb box)</t>
+          <t>Golden Harvest White Rice (2 lb bag)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -4437,22 +4437,22 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="J71" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K71" s="5" t="n">
-        <v>3.49</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>rice-sb-white</t>
+          <t>rice-sb-brown</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -4467,7 +4467,7 @@
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics White Rice (2 lb bag)</t>
+          <t>EveryDay Basics Brown Rice (2 lb bag)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -4495,19 +4495,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K72" s="5" t="n">
-        <v>2.99</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>rice-brand-white</t>
+          <t>rice-brand-brown-org</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -4522,7 +4522,7 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest White Rice (2 lb bag)</t>
+          <t>Golden Harvest Organic Brown Rice (2 lb bag)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -4550,19 +4550,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J73" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K73" s="5" t="n">
-        <v>3.99</v>
+        <v>5.49</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>rice-sb-brown</t>
+          <t>cereal-sb-corn</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -4572,12 +4572,12 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>Cereal</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Brown Rice (2 lb bag)</t>
+          <t>EveryDay Basics Corn Flakes (14 oz box)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -4605,19 +4605,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J74" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K74" s="5" t="n">
-        <v>3.49</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>rice-brand-brown-org</t>
+          <t>cereal-brand-frosted</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -4627,17 +4627,17 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Rice</t>
+          <t>Cereal</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Organic Brown Rice (2 lb bag)</t>
+          <t>Pinnacle Foods Frosted Corn Flakes (14 oz box)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Golden Harvest</t>
+          <t>Pinnacle Foods</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -4647,7 +4647,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -4660,19 +4660,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J75" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K75" s="5" t="n">
-        <v>5.49</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>cereal-sb-corn</t>
+          <t>cereal-sb-bran</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Corn Flakes (14 oz box)</t>
+          <t>EveryDay Basics Bran Flakes (14 oz box)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -4715,19 +4715,19 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J76" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K76" s="5" t="n">
-        <v>2.99</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>cereal-brand-frosted</t>
+          <t>cereal-brand-bran-org</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Frosted Corn Flakes (14 oz box)</t>
+          <t>Pinnacle Foods Organic Bran Flakes (14 oz box)</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -4757,7 +4757,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -4770,34 +4770,34 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="J77" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K77" s="5" t="n">
-        <v>4.49</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>cereal-sb-bran</t>
+          <t>oil-sb-reg</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Bakery &amp; Grains</t>
+          <t>Pantry &amp; Condiments</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Cereal</t>
+          <t>Olive Oil</t>
         </is>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Bran Flakes (14 oz box)</t>
+          <t>EveryDay Basics Olive Oil (16.9 oz)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
@@ -4822,42 +4822,42 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J78" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K78" s="5" t="n">
-        <v>3.49</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>cereal-brand-bran-org</t>
+          <t>oil-brand-evoo</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Bakery &amp; Grains</t>
+          <t>Pantry &amp; Condiments</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Cereal</t>
+          <t>Olive Oil</t>
         </is>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Organic Bran Flakes (14 oz box)</t>
+          <t>Golden Harvest Extra Virgin Olive Oil (16.9 oz)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Pinnacle Foods</t>
+          <t>Golden Harvest</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -4877,22 +4877,22 @@
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J79" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K79" s="5" t="n">
-        <v>5.99</v>
+        <v>8.99</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>oil-sb-reg</t>
+          <t>oil-sb-organic</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Olive Oil (16.9 oz)</t>
+          <t>EveryDay Basics Organic Extra Virgin Olive Oil (16.9 oz)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -4922,7 +4922,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="I80" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="J80" s="7" t="inlineStr">
@@ -4941,13 +4941,13 @@
         </is>
       </c>
       <c r="K80" s="5" t="n">
-        <v>5.99</v>
+        <v>10.99</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>oil-brand-evoo</t>
+          <t>oil-brand-organic-estate</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -4962,7 +4962,7 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Extra Virgin Olive Oil (16.9 oz)</t>
+          <t>Golden Harvest Organic Estate-Grown Olive Oil (16.9 oz)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
@@ -4977,17 +4977,17 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Sustainably Harvested</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="J81" s="7" t="inlineStr">
@@ -4996,13 +4996,13 @@
         </is>
       </c>
       <c r="K81" s="5" t="n">
-        <v>8.99</v>
+        <v>14.99</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>oil-sb-organic</t>
+          <t>tomcan-sb-reg</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -5012,12 +5012,12 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Olive Oil</t>
+          <t>Canned Tomatoes</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Organic Extra Virgin Olive Oil (16.9 oz)</t>
+          <t>EveryDay Basics Diced Tomatoes (28 oz can)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -5042,22 +5042,22 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="J82" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K82" s="5" t="n">
-        <v>10.99</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>oil-brand-organic-estate</t>
+          <t>tomcan-brand-reg</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -5067,12 +5067,12 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Olive Oil</t>
+          <t>Canned Tomatoes</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Organic Estate-Grown Olive Oil (16.9 oz)</t>
+          <t>Golden Harvest Diced Tomatoes (28 oz can)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -5087,32 +5087,32 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>Sustainably Harvested</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="J83" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K83" s="5" t="n">
-        <v>14.99</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>tomcan-sb-reg</t>
+          <t>tomcan-sb-organic</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -5127,7 +5127,7 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Diced Tomatoes (28 oz can)</t>
+          <t>EveryDay Basics Organic Diced Tomatoes (28 oz can)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
@@ -5142,7 +5142,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -5161,13 +5161,13 @@
         </is>
       </c>
       <c r="K84" s="5" t="n">
-        <v>1.49</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>tomcan-brand-reg</t>
+          <t>tomcan-brand-organic-sm</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -5182,7 +5182,7 @@
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Diced Tomatoes (28 oz can)</t>
+          <t>Golden Harvest Organic San Marzano Diced Tomatoes (28 oz can)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
@@ -5197,7 +5197,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -5207,7 +5207,7 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="J85" s="4" t="inlineStr">
@@ -5216,13 +5216,13 @@
         </is>
       </c>
       <c r="K85" s="5" t="n">
-        <v>2.29</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>tomcan-sb-organic</t>
+          <t>pb-sb-reg</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -5232,12 +5232,12 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Canned Tomatoes</t>
+          <t>Peanut Butter</t>
         </is>
       </c>
       <c r="D86" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Organic Diced Tomatoes (28 oz can)</t>
+          <t>EveryDay Basics Peanut Butter (16 oz jar)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -5262,12 +5262,12 @@
       </c>
       <c r="I86" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="J86" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>USA (Georgia)</t>
+        </is>
+      </c>
+      <c r="J86" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K86" s="5" t="n">
@@ -5277,7 +5277,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>tomcan-brand-organic-sm</t>
+          <t>pb-brand-reg</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -5287,17 +5287,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Canned Tomatoes</t>
+          <t>Peanut Butter</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>Golden Harvest Organic San Marzano Diced Tomatoes (28 oz can)</t>
+          <t>Pinnacle Foods Peanut Butter (16 oz jar)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Golden Harvest</t>
+          <t>Pinnacle Foods</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -5317,22 +5317,22 @@
       </c>
       <c r="I87" s="2" t="inlineStr">
         <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="J87" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>USA (Georgia)</t>
+        </is>
+      </c>
+      <c r="J87" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K87" s="5" t="n">
-        <v>4.49</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>pb-sb-reg</t>
+          <t>pb-sb-natural</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -5347,7 +5347,7 @@
       </c>
       <c r="D88" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Peanut Butter (16 oz jar)</t>
+          <t>EveryDay Basics Natural Peanut Butter, No Sugar Added (16 oz jar)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
@@ -5375,19 +5375,19 @@
           <t>USA (Georgia)</t>
         </is>
       </c>
-      <c r="J88" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="J88" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K88" s="5" t="n">
-        <v>2.99</v>
+        <v>4.49</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>pb-brand-reg</t>
+          <t>pb-brand-natural-org</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Peanut Butter (16 oz jar)</t>
+          <t>Pinnacle Foods Organic Natural Peanut Butter (16 oz jar)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -5417,7 +5417,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -5430,19 +5430,19 @@
           <t>USA (Georgia)</t>
         </is>
       </c>
-      <c r="J89" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="J89" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K89" s="5" t="n">
-        <v>4.29</v>
+        <v>6.49</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>pb-sb-natural</t>
+          <t>coffee-sb-std</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
@@ -5452,12 +5452,12 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Peanut Butter</t>
+          <t>Coffee</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Natural Peanut Butter, No Sugar Added (16 oz jar)</t>
+          <t>EveryDay Basics Ground Coffee (12 oz bag)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
@@ -5477,27 +5477,27 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Standard Sourcing</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
         <is>
-          <t>USA (Georgia)</t>
-        </is>
-      </c>
-      <c r="J90" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K90" s="5" t="n">
-        <v>4.49</v>
+        <v>6.99</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>pb-brand-natural-org</t>
+          <t>coffee-brand-std</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -5507,12 +5507,12 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Peanut Butter</t>
+          <t>Coffee</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Organic Natural Peanut Butter (16 oz jar)</t>
+          <t>Pinnacle Foods Ground Coffee (12 oz bag)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -5527,32 +5527,32 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Standard Sourcing</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>USA (Georgia)</t>
-        </is>
-      </c>
-      <c r="J91" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
       <c r="K91" s="5" t="n">
-        <v>6.49</v>
+        <v>8.99</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>coffee-sb-std</t>
+          <t>coffee-sb-ft</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -5567,7 +5567,7 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Ground Coffee (12 oz bag)</t>
+          <t>EveryDay Basics Fair Trade Ground Coffee (12 oz bag)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -5587,12 +5587,12 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Standard Sourcing</t>
+          <t>Fair-Trade Certified</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="J92" s="4" t="inlineStr">
@@ -5601,13 +5601,13 @@
         </is>
       </c>
       <c r="K92" s="5" t="n">
-        <v>6.99</v>
+        <v>10.49</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>coffee-brand-std</t>
+          <t>coffee-brand-ft-org</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -5622,7 +5622,7 @@
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Ground Coffee (12 oz bag)</t>
+          <t>Pinnacle Foods Fair Trade Organic Ground Coffee (12 oz bag)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
@@ -5637,17 +5637,17 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Standard Sourcing</t>
+          <t>Fair-Trade Certified</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Ethiopia</t>
         </is>
       </c>
       <c r="J93" s="4" t="inlineStr">
@@ -5656,28 +5656,28 @@
         </is>
       </c>
       <c r="K93" s="5" t="n">
-        <v>8.99</v>
+        <v>13.99</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>coffee-sb-ft</t>
+          <t>choc-sb-milk</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Pantry &amp; Condiments</t>
+          <t>Snacks &amp; Beverages</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Chocolate Bar</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Fair Trade Ground Coffee (12 oz bag)</t>
+          <t>EveryDay Basics Milk Chocolate Bar (3.5 oz)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
@@ -5697,42 +5697,42 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Fair-Trade Certified</t>
+          <t>Standard Sourcing</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="J94" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Cote d'Ivoire</t>
+        </is>
+      </c>
+      <c r="J94" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K94" s="5" t="n">
-        <v>10.49</v>
+        <v>1.99</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>coffee-brand-ft-org</t>
+          <t>choc-brand-milk</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Pantry &amp; Condiments</t>
+          <t>Snacks &amp; Beverages</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Coffee</t>
+          <t>Chocolate Bar</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Fair Trade Organic Ground Coffee (12 oz bag)</t>
+          <t>Pinnacle Foods Milk Chocolate Bar (3.5 oz)</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -5747,32 +5747,32 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Fair-Trade Certified</t>
+          <t>Standard Sourcing</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
-        </is>
-      </c>
-      <c r="J95" s="4" t="inlineStr">
-        <is>
-          <t>A</t>
+          <t>Cote d'Ivoire</t>
+        </is>
+      </c>
+      <c r="J95" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K95" s="5" t="n">
-        <v>13.99</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>choc-sb-milk</t>
+          <t>choc-sb-dark-ft</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5787,7 +5787,7 @@
       </c>
       <c r="D96" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Milk Chocolate Bar (3.5 oz)</t>
+          <t>EveryDay Basics Fair Trade Dark Chocolate Bar 70% (3.5 oz)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -5807,27 +5807,27 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Standard Sourcing</t>
+          <t>Fair-Trade Certified</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr">
         <is>
-          <t>Cote d'Ivoire</t>
-        </is>
-      </c>
-      <c r="J96" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="J96" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K96" s="5" t="n">
-        <v>1.99</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>choc-brand-milk</t>
+          <t>choc-brand-dark-ft-org</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5842,7 +5842,7 @@
       </c>
       <c r="D97" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Milk Chocolate Bar (3.5 oz)</t>
+          <t>Pinnacle Foods Fair Trade Organic Dark Chocolate Bar 70% (3.5 oz)</t>
         </is>
       </c>
       <c r="E97" s="2" t="inlineStr">
@@ -5857,32 +5857,32 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Standard Sourcing</t>
+          <t>Fair-Trade Certified</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr">
         <is>
-          <t>Cote d'Ivoire</t>
-        </is>
-      </c>
-      <c r="J97" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="J97" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K97" s="5" t="n">
-        <v>2.99</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>choc-sb-dark-ft</t>
+          <t>chips-sb-reg</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -5892,12 +5892,12 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>Chocolate Bar</t>
+          <t>Potato Chips</t>
         </is>
       </c>
       <c r="D98" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Fair Trade Dark Chocolate Bar 70% (3.5 oz)</t>
+          <t>EveryDay Basics Potato Chips (8 oz bag)</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -5917,27 +5917,27 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Fair-Trade Certified</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr">
         <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="J98" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>USA (Idaho)</t>
+        </is>
+      </c>
+      <c r="J98" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K98" s="5" t="n">
-        <v>3.49</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>choc-brand-dark-ft-org</t>
+          <t>chips-brand-reg</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -5947,12 +5947,12 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Chocolate Bar</t>
+          <t>Potato Chips</t>
         </is>
       </c>
       <c r="D99" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Fair Trade Organic Dark Chocolate Bar 70% (3.5 oz)</t>
+          <t>Pinnacle Foods Potato Chips (8 oz bag)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
@@ -5967,32 +5967,32 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Fair-Trade Certified</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr">
         <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="J99" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>USA (Idaho)</t>
+        </is>
+      </c>
+      <c r="J99" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
         </is>
       </c>
       <c r="K99" s="5" t="n">
-        <v>4.99</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>chips-sb-reg</t>
+          <t>chips-sb-reducedfat</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -6007,7 +6007,7 @@
       </c>
       <c r="D100" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Potato Chips (8 oz bag)</t>
+          <t>EveryDay Basics Reduced Fat Potato Chips (8 oz bag)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
@@ -6035,19 +6035,19 @@
           <t>USA (Idaho)</t>
         </is>
       </c>
-      <c r="J100" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="J100" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K100" s="5" t="n">
-        <v>2.49</v>
+        <v>3.29</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>chips-brand-reg</t>
+          <t>chips-brand-avocado-org</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Potato Chips (8 oz bag)</t>
+          <t>Pinnacle Foods Organic Potato Chips, Avocado Oil (8 oz bag)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -6090,19 +6090,19 @@
           <t>USA (Idaho)</t>
         </is>
       </c>
-      <c r="J101" s="9" t="inlineStr">
-        <is>
-          <t>E</t>
+      <c r="J101" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="K101" s="5" t="n">
-        <v>3.79</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>chips-sb-reducedfat</t>
+          <t>oj-sb-conc</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -6112,12 +6112,12 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Potato Chips</t>
+          <t>Orange Juice</t>
         </is>
       </c>
       <c r="D102" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Reduced Fat Potato Chips (8 oz bag)</t>
+          <t>EveryDay Basics Orange Juice, From Concentrate (64 oz)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -6142,22 +6142,22 @@
       </c>
       <c r="I102" s="2" t="inlineStr">
         <is>
-          <t>USA (Idaho)</t>
-        </is>
-      </c>
-      <c r="J102" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>USA (Florida)</t>
+        </is>
+      </c>
+      <c r="J102" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K102" s="5" t="n">
-        <v>3.29</v>
+        <v>2.99</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>chips-brand-avocado-org</t>
+          <t>oj-brand-conc</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -6167,17 +6167,17 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Potato Chips</t>
+          <t>Orange Juice</t>
         </is>
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>Pinnacle Foods Organic Potato Chips, Avocado Oil (8 oz bag)</t>
+          <t>Sunrise Farms Orange Juice, From Concentrate (64 oz)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Pinnacle Foods</t>
+          <t>Sunrise Farms</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -6187,7 +6187,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -6197,22 +6197,22 @@
       </c>
       <c r="I103" s="2" t="inlineStr">
         <is>
-          <t>USA (Idaho)</t>
-        </is>
-      </c>
-      <c r="J103" s="8" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>USA (Florida)</t>
+        </is>
+      </c>
+      <c r="J103" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
         </is>
       </c>
       <c r="K103" s="5" t="n">
-        <v>4.99</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>oj-sb-conc</t>
+          <t>oj-sb-nfc</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>EveryDay Basics Orange Juice, From Concentrate (64 oz)</t>
+          <t>EveryDay Basics Not-From-Concentrate Orange Juice (64 oz)</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
@@ -6255,19 +6255,19 @@
           <t>USA (Florida)</t>
         </is>
       </c>
-      <c r="J104" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="J104" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K104" s="5" t="n">
-        <v>2.99</v>
+        <v>4.99</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>oj-brand-conc</t>
+          <t>oj-brand-nfc-org</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="D105" s="3" t="inlineStr">
         <is>
-          <t>Sunrise Farms Orange Juice, From Concentrate (64 oz)</t>
+          <t>Sunrise Farms Organic Not-From-Concentrate Orange Juice (64 oz)</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -6310,127 +6310,17 @@
           <t>USA (Florida)</t>
         </is>
       </c>
-      <c r="J105" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
+      <c r="J105" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="K105" s="5" t="n">
-        <v>4.29</v>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>oj-sb-nfc</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr">
-        <is>
-          <t>Snacks &amp; Beverages</t>
-        </is>
-      </c>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>Orange Juice</t>
-        </is>
-      </c>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>EveryDay Basics Not-From-Concentrate Orange Juice (64 oz)</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>EveryDay Basics</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>Off-Brand</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H106" s="2" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="I106" s="2" t="inlineStr">
-        <is>
-          <t>USA (Florida)</t>
-        </is>
-      </c>
-      <c r="J106" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="K106" s="5" t="n">
-        <v>4.99</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>oj-brand-nfc-org</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="inlineStr">
-        <is>
-          <t>Snacks &amp; Beverages</t>
-        </is>
-      </c>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>Orange Juice</t>
-        </is>
-      </c>
-      <c r="D107" s="3" t="inlineStr">
-        <is>
-          <t>Sunrise Farms Organic Not-From-Concentrate Orange Juice (64 oz)</t>
-        </is>
-      </c>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>Sunrise Farms</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>Brand</t>
-        </is>
-      </c>
-      <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H107" s="2" t="inlineStr">
-        <is>
-          <t>Standard</t>
-        </is>
-      </c>
-      <c r="I107" s="2" t="inlineStr">
-        <is>
-          <t>USA (Florida)</t>
-        </is>
-      </c>
-      <c r="J107" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="K107" s="5" t="n">
         <v>6.99</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K107"/>
+  <autoFilter ref="A1:K105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6552,7 +6442,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>European front-of-pack nutrition grade, A (healthiest) to E (least healthy), color-coded to the official scheme. Reflects the food itself, not its brand/organic/ethics status — e.g. a raw apple is grade A whether organic or not. Varies within a product type only where a genuinely different formulation exists (e.g. plain vs. sweetened yogurt, white vs. whole-wheat bread).</t>
+          <t>European front-of-pack nutrition grade, A (healthiest) to E (least healthy), color-coded to the official scheme. Reflects the food itself, not its brand/organic/ethics status — e.g. a raw apple is grade A whether organic or not. Varies within a product type only where a genuinely different formulation exists (e.g. plain corn flakes vs. frosted, white vs. whole-wheat bread).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire in real photos for all 13 new product types, add cart icon
Replaces the remaining 36 placeholder SVGs (Pork Chops, Tortillas, Oats,
Pasta Sauce, Honey, Soda, Tofu, Hummus, Frozen Pizza) with real photos
Gavin dropped into Item Pictures/, mapped by price rank via an extended
apply_new_item_photos.py. All 156 catalog items now have real photos.

Also adds a shopping-cart icon next to the basket link, with basket.js
updated to target the count text specifically so the icon survives AJAX
basket updates.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog-design.xlsx
+++ b/catalog-design.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalog'!$A$1:$K$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalog'!$A$1:$K$157</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K105"/>
+  <dimension ref="A1:K157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -6319,8 +6319,2868 @@
         <v>6.99</v>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>onions-sb-conv</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Onions</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Yellow Onions (3 lb bag)</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>USA (Oregon)</t>
+        </is>
+      </c>
+      <c r="J106" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K106" s="5" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>onions-brand-conv</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Onions</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Farms Yellow Onions (3 lb bag)</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Sunrise Farms</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>USA (Oregon)</t>
+        </is>
+      </c>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K107" s="5" t="n">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>onions-sb-organic</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Onions</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Yellow Onions (3 lb bag)</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Organic Farming</t>
+        </is>
+      </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>USA (Oregon)</t>
+        </is>
+      </c>
+      <c r="J108" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K108" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>onions-brand-organic</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Onions</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Farms Organic Yellow Onions (3 lb bag)</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>Sunrise Farms</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Organic Farming</t>
+        </is>
+      </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>USA (Oregon)</t>
+        </is>
+      </c>
+      <c r="J109" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K109" s="5" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>carrots-sb-conv</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Carrots</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Carrots (2 lb bag)</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>USA (California)</t>
+        </is>
+      </c>
+      <c r="J110" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>carrots-brand-conv</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Carrots</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Farms Carrots (2 lb bag)</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>Sunrise Farms</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Conventional</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>USA (California)</t>
+        </is>
+      </c>
+      <c r="J111" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="n">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>carrots-sb-organic</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Carrots</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Carrots (2 lb bag)</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Organic Farming</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>USA (California)</t>
+        </is>
+      </c>
+      <c r="J112" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>carrots-brand-organic</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Carrots</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Farms Organic Carrots (2 lb bag)</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>Sunrise Farms</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Organic Farming</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>USA (California)</t>
+        </is>
+      </c>
+      <c r="J113" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K113" s="5" t="n">
+        <v>4.29</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>avocados-sb-imp</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Avocados</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Avocados (4 ct bag)</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="J114" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K114" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>avocados-brand-imp</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Avocados</t>
+        </is>
+      </c>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Farms Avocados (4 ct bag)</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>Sunrise Farms</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Imported</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="J115" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K115" s="5" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>avocados-sb-local-org</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Avocados</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Local Organic Avocados (4 ct bag)</t>
+        </is>
+      </c>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Locally Grown</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>USA (California)</t>
+        </is>
+      </c>
+      <c r="J116" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K116" s="5" t="n">
+        <v>6.49</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>avocados-brand-local-org</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Avocados</t>
+        </is>
+      </c>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Farms Local Organic Avocados (4 ct bag)</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>Sunrise Farms</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Locally Grown</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>USA (California)</t>
+        </is>
+      </c>
+      <c r="J117" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K117" s="5" t="n">
+        <v>7.99</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>sourcream-sb-conv</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Sour Cream</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Sour Cream (16 oz)</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Conventional Dairy</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>USA (Wisconsin)</t>
+        </is>
+      </c>
+      <c r="J118" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K118" s="5" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>sourcream-brand-conv</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Sour Cream</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>Green Pasture Co. Sour Cream (16 oz)</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>Green Pasture Co.</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>Conventional Dairy</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>USA (Wisconsin)</t>
+        </is>
+      </c>
+      <c r="J119" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K119" s="5" t="n">
+        <v>2.79</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>sourcream-sb-organic</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Sour Cream</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Sour Cream (16 oz)</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Pasture-Raised</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>USA (Vermont)</t>
+        </is>
+      </c>
+      <c r="J120" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K120" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>sourcream-brand-organic</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>Dairy &amp; Eggs</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Sour Cream</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>Green Pasture Co. Organic Sour Cream (16 oz)</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>Green Pasture Co.</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Pasture-Raised</t>
+        </is>
+      </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>USA (Vermont)</t>
+        </is>
+      </c>
+      <c r="J121" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K121" s="5" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>pork-sb-factory</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>Meat &amp; Seafood</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Pork Chops</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Pork Chops (1 lb)</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Factory-Farmed</t>
+        </is>
+      </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J122" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K122" s="5" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>pork-brand-factory</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Meat &amp; Seafood</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Pork Chops</t>
+        </is>
+      </c>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>Heritage Range Pork Chops (1 lb)</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>Heritage Range</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>Factory-Farmed</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J123" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K123" s="5" t="n">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>pork-sb-freerange</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Meat &amp; Seafood</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Pork Chops</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Free-Range Pork Chops (1 lb)</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Free-Range</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J124" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K124" s="5" t="n">
+        <v>7.49</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>pork-brand-freerange-org</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Meat &amp; Seafood</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Pork Chops</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>Heritage Range Organic Free-Range Pork Chops (1 lb)</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>Heritage Range</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>Free-Range</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J125" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K125" s="5" t="n">
+        <v>9.99</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>tortillas-sb-flour</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Tortillas</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Flour Tortillas (10 ct)</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J126" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K126" s="5" t="n">
+        <v>2.29</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>tortillas-brand-flour</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Tortillas</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Flour Tortillas (10 ct)</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J127" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K127" s="5" t="n">
+        <v>3.29</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>tortillas-sb-wheat</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Tortillas</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Whole Wheat Tortillas (10 ct)</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J128" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K128" s="5" t="n">
+        <v>2.79</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>tortillas-brand-wheat-org</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Tortillas</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Organic Whole Wheat Tortillas (10 ct)</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J129" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K129" s="5" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>oats-sb-rolled</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Oats</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Rolled Oats (18 oz)</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J130" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K130" s="5" t="n">
+        <v>2.49</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>oats-brand-rolled</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Oats</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Rolled Oats (18 oz)</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J131" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K131" s="5" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>oats-sb-organic</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>Oats</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Rolled Oats (18 oz)</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G132" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J132" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K132" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>oats-brand-organic</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>Bakery &amp; Grains</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>Oats</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Organic Rolled Oats (18 oz)</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J133" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K133" s="5" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>sauce-sb-reg</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Marinara Pasta Sauce (24 oz jar)</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G134" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J134" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K134" s="5" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>sauce-brand-reg</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D135" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Marinara Pasta Sauce (24 oz jar)</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J135" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K135" s="5" t="n">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>sauce-sb-organic</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Marinara Pasta Sauce (24 oz jar)</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J136" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K136" s="5" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>sauce-brand-organic-sm</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Pasta Sauce</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Organic San Marzano Pasta Sauce (24 oz jar)</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>Italy</t>
+        </is>
+      </c>
+      <c r="J137" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K137" s="5" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>honey-sb-std</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Honey</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Honey (12 oz)</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="J138" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K138" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>honey-brand-std</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Honey</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Honey (12 oz)</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="J139" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K139" s="5" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>honey-sb-raw-local</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Honey</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Raw Local Honey (12 oz)</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Raw &amp; Unfiltered</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>USA (Vermont)</t>
+        </is>
+      </c>
+      <c r="J140" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K140" s="5" t="n">
+        <v>6.99</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>honey-brand-raw-local-org</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>Pantry &amp; Condiments</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Honey</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>Golden Harvest Organic Raw Local Honey (12 oz)</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>Golden Harvest</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>Raw &amp; Unfiltered</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>USA (Vermont)</t>
+        </is>
+      </c>
+      <c r="J141" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K141" s="5" t="n">
+        <v>8.99</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>soda-sb-reg</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Soda</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Cola (12-pack cans)</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J142" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="K142" s="5" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>soda-brand-reg</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Soda</t>
+        </is>
+      </c>
+      <c r="D143" s="3" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods Cola (12-pack cans)</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J143" s="9" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="K143" s="5" t="n">
+        <v>5.99</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>soda-sb-diet</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Soda</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Diet Cola (12-pack cans)</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J144" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K144" s="5" t="n">
+        <v>4.99</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>soda-brand-diet</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Soda</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods Diet Cola (12-pack cans)</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods</t>
+        </is>
+      </c>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J145" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K145" s="5" t="n">
+        <v>6.49</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>tofu-sb-std</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Tofu</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Firm Tofu (14 oz)</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F146" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Standard Soybeans</t>
+        </is>
+      </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J146" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K146" s="5" t="n">
+        <v>1.99</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>tofu-brand-std</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Tofu</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods Firm Tofu (14 oz)</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods</t>
+        </is>
+      </c>
+      <c r="F147" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Standard Soybeans</t>
+        </is>
+      </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J147" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K147" s="5" t="n">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>tofu-sb-organic</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Tofu</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Non-GMO Firm Tofu (14 oz)</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Organic Non-GMO Soybeans</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>USA (Iowa)</t>
+        </is>
+      </c>
+      <c r="J148" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K148" s="5" t="n">
+        <v>3.49</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>tofu-brand-organic</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Tofu</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods Organic Non-GMO Firm Tofu (14 oz)</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>Organic Non-GMO Soybeans</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="J149" s="4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="K149" s="5" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>hummus-sb-reg</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Hummus</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Classic Hummus (10 oz)</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J150" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="n">
+        <v>2.99</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>hummus-brand-reg</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Hummus</t>
+        </is>
+      </c>
+      <c r="D151" s="3" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods Classic Hummus (10 oz)</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods</t>
+        </is>
+      </c>
+      <c r="F151" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J151" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K151" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>hummus-sb-organic</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Hummus</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Classic Hummus (10 oz)</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F152" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J152" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K152" s="5" t="n">
+        <v>4.49</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>hummus-brand-organic</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>Plant-Based &amp; Vegetarian</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="inlineStr">
+        <is>
+          <t>Hummus</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods Organic Classic Hummus (10 oz)</t>
+        </is>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>Terra Verde Foods</t>
+        </is>
+      </c>
+      <c r="F153" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G153" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J153" s="6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="K153" s="5" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>pizza-sb-reg</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>Frozen Pizza</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Frozen Pepperoni Pizza (12 in)</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J154" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K154" s="5" t="n">
+        <v>3.99</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>pizza-brand-reg</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Frozen Pizza</t>
+        </is>
+      </c>
+      <c r="D155" s="3" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods Frozen Pepperoni Pizza (12 in)</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J155" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="K155" s="5" t="n">
+        <v>5.49</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>pizza-sb-organic</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Frozen Pizza</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>EveryDay Basics Organic Frozen Margherita Pizza (12 in)</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>EveryDay Basics</t>
+        </is>
+      </c>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>Off-Brand</t>
+        </is>
+      </c>
+      <c r="G156" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J156" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K156" s="5" t="n">
+        <v>6.49</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>pizza-brand-organic</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Frozen</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Frozen Pizza</t>
+        </is>
+      </c>
+      <c r="D157" s="3" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods Organic Frozen Margherita Pizza (12 in)</t>
+        </is>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>Pinnacle Foods</t>
+        </is>
+      </c>
+      <c r="F157" s="2" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="G157" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="J157" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="K157" s="5" t="n">
+        <v>7.99</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K105"/>
+  <autoFilter ref="A1:K157"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6469,7 +9329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6541,7 +9401,7 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Meat &amp; Seafood</t>
+          <t>Frozen</t>
         </is>
       </c>
       <c r="B4" s="13">
@@ -6560,7 +9420,7 @@
     <row r="5">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Pantry &amp; Condiments</t>
+          <t>Meat &amp; Seafood</t>
         </is>
       </c>
       <c r="B5" s="13">
@@ -6579,7 +9439,7 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Produce</t>
+          <t>Pantry &amp; Condiments</t>
         </is>
       </c>
       <c r="B6" s="13">
@@ -6598,7 +9458,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Snacks &amp; Beverages</t>
+          <t>Plant-Based &amp; Vegetarian</t>
         </is>
       </c>
       <c r="B7" s="13">
@@ -6615,13 +9475,51 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Produce</t>
+        </is>
+      </c>
+      <c r="B8" s="13">
+        <f>COUNTIF(Catalog!B:B,A8)</f>
+        <v/>
+      </c>
+      <c r="C8" s="14">
+        <f>AVERAGEIFS(Catalog!K:K,Catalog!B:B,A8,Catalog!F:F,"Off-Brand")</f>
+        <v/>
+      </c>
+      <c r="D8" s="14">
+        <f>AVERAGEIFS(Catalog!K:K,Catalog!B:B,A8,Catalog!F:F,"Brand")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Snacks &amp; Beverages</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>COUNTIF(Catalog!B:B,A9)</f>
+        <v/>
+      </c>
+      <c r="C9" s="14">
+        <f>AVERAGEIFS(Catalog!K:K,Catalog!B:B,A9,Catalog!F:F,"Off-Brand")</f>
+        <v/>
+      </c>
+      <c r="D9" s="14">
+        <f>AVERAGEIFS(Catalog!K:K,Catalog!B:B,A9,Catalog!F:F,"Brand")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B8" s="15">
-        <f>SUM(B2:B7)</f>
+      <c r="B10" s="15">
+        <f>SUM(B2:B9)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch budget conditions and currency display to euros
Budget conditions are now low=30/medium=50/high=70 EUR (was
20/40/70 USD). Renamed $ to € throughout the live views and AJAX
basket updates, and renamed the CSV export's _usd columns to _eur
to match, with the analysis script and catalog-design.xlsx updated
to follow.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/catalog-design.xlsx
+++ b/catalog-design.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="€#,##0.00"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -9314,7 +9314,7 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Fictional USD retail price. Within any matched pair, Off-Brand &lt; Brand, and conventional &lt; organic/ethically-sourced.</t>
+          <t>Fictional EUR retail price. Within any matched pair, Off-Brand &lt; Brand, and conventional &lt; organic/ethically-sourced.</t>
         </is>
       </c>
     </row>

</xml_diff>